<commit_message>
feat(fleet): render local OSM street maps in trip reports and complete audit evidence
</commit_message>
<xml_diff>
--- a/docs/fleet-assets-audit/evidence/PKG-02B/implementation/final-audit-20260926/pw-track-veh-trips-2026-09-23-to-2026-09-24.xlsx
+++ b/docs/fleet-assets-audit/evidence/PKG-02B/implementation/final-audit-20260926/pw-track-veh-trips-2026-09-23-to-2026-09-24.xlsx
@@ -5,7 +5,7 @@
     <sheet name="Trips" sheetId="1" r:id="sheet1"/>
     <sheet name="Events" sheetId="2" r:id="sheet2"/>
     <sheet name="Report notes" sheetId="3" r:id="sheet3"/>
-    <sheet name="Journey sketches" sheetId="4" r:id="sheet4"/>
+    <sheet name="Journey maps" sheetId="4" r:id="sheet4"/>
   </sheets>
   <calcPr fullCalcOnLoad="1"/>
 </workbook>
@@ -73,7 +73,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>7</xdr:row>
+      <xdr:row>8</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="7429500" cy="3143250"/>
@@ -104,7 +104,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>30</xdr:row>
+      <xdr:row>32</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="7429500" cy="3143250"/>
@@ -850,7 +850,7 @@
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Generated 26 Sep 2026, 10:28 pm by Demo Admin</t>
+          <t xml:space="preserve">Generated 26 Sep 2026, 11:23 pm by Demo Admin</t>
         </is>
       </c>
     </row>
@@ -951,7 +951,7 @@
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Position sketches only. Lines are not verified roads; gaps remain unknown.</t>
+          <t xml:space="preserve">Recorded positions over the available local map. Lines are not verified roads; gaps remain unknown.</t>
         </is>
       </c>
     </row>
@@ -970,7 +970,13 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="24" customHeight="1"/>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Local street map · New Zealand · data 2026-09-23. © OpenStreetMap contributors · ODbL · openstreetmap.org/copyright</t>
+        </is>
+      </c>
+    </row>
     <row r="9" ht="24" customHeight="1"/>
     <row r="10" ht="24" customHeight="1"/>
     <row r="11" ht="24" customHeight="1"/>
@@ -989,30 +995,36 @@
     <row r="24" ht="24" customHeight="1"/>
     <row r="25" ht="24" customHeight="1"/>
     <row r="26" ht="24" customHeight="1"/>
-    <row r="27" ht="24" customHeight="1">
-      <c r="A27" s="0" t="inlineStr">
+    <row r="27" ht="24" customHeight="1"/>
+    <row r="28" ht="24" customHeight="1">
+      <c r="A28" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Tracker: Queclink</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="24" customHeight="1"/>
-    <row r="29" ht="24" customHeight="1">
-      <c r="A29" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Trip #3 · Thu 24 Sep 2026 · 12:02 am–12:14 am</t>
-        </is>
-      </c>
-    </row>
+    <row r="29" ht="24" customHeight="1"/>
     <row r="30" ht="24" customHeight="1">
       <c r="A30" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">Trip #3 · Thu 24 Sep 2026 · 12:02 am–12:14 am</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="24" customHeight="1">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">QA Main Site → Hospital outpatients, Grafton</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="24" customHeight="1"/>
-    <row r="32" ht="24" customHeight="1"/>
+    <row r="32" ht="24" customHeight="1">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Local street map · New Zealand · data 2026-09-23. © OpenStreetMap contributors · ODbL · openstreetmap.org/copyright</t>
+        </is>
+      </c>
+    </row>
     <row r="33" ht="24" customHeight="1"/>
     <row r="34" ht="24" customHeight="1"/>
     <row r="35" ht="24" customHeight="1"/>
@@ -1030,26 +1042,30 @@
     <row r="47" ht="24" customHeight="1"/>
     <row r="48" ht="24" customHeight="1"/>
     <row r="49" ht="24" customHeight="1"/>
-    <row r="50" ht="24" customHeight="1">
-      <c r="A50" s="0" t="inlineStr">
+    <row r="50" ht="24" customHeight="1"/>
+    <row r="51" ht="24" customHeight="1"/>
+    <row r="52" ht="24" customHeight="1">
+      <c r="A52" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Tracker: Queclink</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="24" customHeight="1"/>
+    <row r="53" ht="24" customHeight="1"/>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="12">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="A6:H6"/>
     <mergeCell ref="A7:H7"/>
-    <mergeCell ref="A27:H27"/>
-    <mergeCell ref="A29:H29"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A28:H28"/>
     <mergeCell ref="A30:H30"/>
-    <mergeCell ref="A50:H50"/>
+    <mergeCell ref="A31:H31"/>
+    <mergeCell ref="A32:H32"/>
+    <mergeCell ref="A52:H52"/>
   </mergeCells>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" paperSize="9" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
fix(fleet): retain trip duration precision in Excel reports
</commit_message>
<xml_diff>
--- a/docs/fleet-assets-audit/evidence/PKG-02B/implementation/final-audit-20260926/pw-track-veh-trips-2026-09-23-to-2026-09-24.xlsx
+++ b/docs/fleet-assets-audit/evidence/PKG-02B/implementation/final-audit-20260926/pw-track-veh-trips-2026-09-23-to-2026-09-24.xlsx
@@ -51,7 +51,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -60,6 +60,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -309,7 +312,7 @@
       <c r="I8" s="0">
         <v>4.2</v>
       </c>
-      <c r="J8" s="0">
+      <c r="J8" s="4">
         <v>15</v>
       </c>
       <c r="K8" s="0">
@@ -372,7 +375,7 @@
       <c r="I9" s="0">
         <v>9.6</v>
       </c>
-      <c r="J9" s="0">
+      <c r="J9" s="4">
         <v>12</v>
       </c>
       <c r="K9" s="0">
@@ -438,7 +441,7 @@
         <f>SUM(I8:I9)</f>
         <v>13.8</v>
       </c>
-      <c r="J10" s="0">
+      <c r="J10" s="4">
         <f>SUM(J8:J9)</f>
         <v>27</v>
       </c>
@@ -850,7 +853,7 @@
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Generated 26 Sep 2026, 11:23 pm by Demo Admin</t>
+          <t xml:space="preserve">Generated 27 Sep 2026, 12:03 am by Demo Admin</t>
         </is>
       </c>
     </row>
@@ -858,47 +861,54 @@
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Distance is the tracker's GPS estimate, not a dashboard odometer reading. Odometer readings keep their own evidence.</t>
+          <t xml:space="preserve">Duration retains recorded seconds as fractional minutes. Cells display two decimals; totals use the unrounded values.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
       <c r="A6" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">Distance is the tracker's GPS estimate, not a dashboard odometer reading. Odometer readings keep their own evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">Coverage is the share of each trip with a recorded position at least every 2 min. Lines between recorded positions are not verified roads.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="48" customHeight="1">
-      <c r="A7" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Behaviour score: 100 − 5 × harsh braking − 3 × harsh acceleration − 3 × other harsh events − 4 × overspeed episodes − 0.5 × idle minutes, from the fleet settings. Scores are withheld below 90% coverage.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">Behaviour score: 100 − 5 × harsh braking − 3 × harsh acceleration − 3 × other harsh events − 4 × overspeed episodes − 0.5 × idle minutes, from the fleet settings. Scores are withheld below 90% coverage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">Human review applies: dismissed events do not deduct points and disputed events withhold the score. Event counts retain the original recorded observations.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overspeed uses the fleet threshold of 100 km/h; road speed limits are not checked.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">Overspeed uses the fleet threshold of 100 km/h; road speed limits are not checked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">A booked driver is not proof of who drove. Drivers are shown as confirmed only after someone confirms them.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A3:H3"/>
@@ -908,6 +918,7 @@
     <mergeCell ref="A8:H8"/>
     <mergeCell ref="A9:H9"/>
     <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A11:H11"/>
   </mergeCells>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" paperSize="9" fitToWidth="1" fitToHeight="0"/>

</xml_diff>